<commit_message>
LØM-app 2.6.2: V5-presentasjoner, formel før levering og hint i regnearket
</commit_message>
<xml_diff>
--- a/pensum/ma01/MA01_Klasseoppgaver_v5.xlsx
+++ b/pensum/ma01/MA01_Klasseoppgaver_v5.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="153">
   <si>
     <t xml:space="preserve">Klasseoppgaver til Markedsføring kapittel 1: Hva er markedsføring? (V5)</t>
   </si>
@@ -182,6 +182,27 @@
     <t xml:space="preserve">e)  Kari sier: «Vi trenger ikke markedsføring, vi har nok å gjøre.» Svar henne i to setninger: én med bokas definisjon, og én med et konkret eksempel fra de seks forespørslene.</t>
   </si>
   <si>
+    <t xml:space="preserve">Formel og begrep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definisjonen av markedsføring, med lønnsomhet som endelig mål (kap. 1, innledningen). Markedsføringsledelse er det overordnede ansvaret for planlegging, iverksetting og evaluering (innledningen).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hint, hvis du står fast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hvem kjøper, og hvorfor?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spør for hver kunde: kjøper de til eget bruk, i næring, for å selge videre, som offentlig forvaltning eller som frivillig organisasjon? Det avgjør hovedmarkedet (slide 10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Virksomheten, ikke eieren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boka plasserer offentlig næringsdrift, også selskaper kommunen eier, i bedriftsmarkedet. Det offentlige markedet er forvaltningen (slide 10).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kilde: Hjertnes, F.: Markedsføring, organisasjon og ledelse for LØM-emnet, kap. 1, innledningen, 1.1 og 1.4.1–1.4.5. Nordlys Elektro AS er en konstruert casebedrift.</t>
   </si>
   <si>
@@ -269,6 +290,21 @@
     <t xml:space="preserve">e)  Fjell har 3 500 fakturerbare timer og ingen rammeavtaler. Bør Mona satse først på boligkunder (forbrukermarkedet) eller små næringskunder (bedriftsmarkedet)? Begrunn, og si hva tilbudet da må ha med.</t>
   </si>
   <si>
+    <t xml:space="preserve">Forbrukere er amatører og mer styrt av følelser; bedriftene kjøper mer rasjonelt (Markedsføring 1.4.5 og 1.4.1). Markedsføringsledelse er Monas ansvar (innledningen).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hvem kjøper til eget bruk?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forbrukermarkedet er enkeltpersoner og husholdninger som kjøper til eget konsum. Bedrifter, kommunen og foreninger hører til andre hovedmarkeder (slide 10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fem P-er, ikke én</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annonser er påvirkning. Produkt, pris, plass og personal er også markedsføring (slide 7). Og noen må eie oppgaven, også med tre ansatte (slide 8).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kilde: Hjertnes, F.: Markedsføring, organisasjon og ledelse for LØM-emnet, kap. 1, innledningen og 1.4; de fem P-ene i kap. 3.5. Fjell Elektro AS er en konstruert casebedrift.</t>
   </si>
   <si>
@@ -353,6 +389,21 @@
     <t xml:space="preserve">e)  Skriv tre ting Ida bør spørre et borettslagsstyre om før hun skriver neste tilbud, og si hvilket av forslagene (1–5) du bygger på.</t>
   </si>
   <si>
+    <t xml:space="preserve">Markedsorientering (1.2.4). Relasjonsmarkedsføring og intern markedsføring i helhetlig markedsorientering (1.2.5).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hvor starter forslaget?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Starter det med det Nordlys har (anlegget, prisen, volumet), eller med det kunden trenger? Det er skillet mellom trinn 3 og 4 i trappa (slide 26–27).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fem stikkord</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Billig og effektivt: produksjon. Best mulig produkt: produkt. Mer volum, flere kjøpere: salg. Kundens behov: marked. Ansatte, relasjoner og samfunn i tillegg: helhetlig.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kilde: Hjertnes, F.: Markedsføring, organisasjon og ledelse for LØM-emnet, kap. 1, 1.2 og 1.2.1–1.2.5. Nordlys Elektro AS er en konstruert casebedrift.</t>
   </si>
   <si>
@@ -414,6 +465,21 @@
   </si>
   <si>
     <t xml:space="preserve">e)  Kan slagordet «Bærekraftig elektro i Oslo øst» stå? Begrunn, og skriv én setning Mona kan bruke i stedet, som er dekket av det Fjell faktisk gjør.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helhetlig markedsorientering: etiske normer og miljøhensyn (1.2.5). Bærekraftig utvikling og lov som minimum (1.2.5.1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tre krav samtidig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Det som loves eksternt, må stemme internt. Relasjoner bygges over tid og gir synergi. Alt skjer innenfor lov, etikk og miljøhensyn (slide 28).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loven er gulvet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lovgivningen er som regel bare minimumsløsninger. Spør: hvilket av Fjells tiltak gjelder det Fjell selger og kjøringen, ikke bare avfallet (slide 29)?</t>
   </si>
   <si>
     <t xml:space="preserve">Kilde: Hjertnes, F.: Markedsføring, organisasjon og ledelse for LØM-emnet, kap. 1, 1.2.5 og 1.2.5.1. Fjell Elektro AS er en konstruert casebedrift.</t>
@@ -426,7 +492,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -493,8 +559,30 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF2F4A6D"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -510,13 +598,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF4F6FA"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFEEF2F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF2F8"/>
+        <bgColor rgb="FFF4F6FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB8954A"/>
+        <bgColor rgb="FF808080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBF6EA"/>
+        <bgColor rgb="FFF4F6FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -569,7 +675,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -642,6 +748,26 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -675,8 +801,8 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF4F6FA"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFFBF6EA"/>
+      <rgbColor rgb="FFEEF2F8"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -690,7 +816,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFF4F6FA"/>
       <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
@@ -704,7 +830,7 @@
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF5E6670"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FFB8954A"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
@@ -1007,7 +1133,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1287,30 +1413,80 @@
       <c r="F29" s="17"/>
       <c r="G29" s="17"/>
     </row>
-    <row r="31" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
+    <row r="30" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
+      <c r="B30" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
+      <c r="G30" s="19"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="20"/>
+    </row>
+    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+    </row>
+    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35" s="22"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="22"/>
+    </row>
+    <row r="37" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="21">
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A14:G14"/>
@@ -1326,8 +1502,12 @@
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A27:G29"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="B34:G34"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A38:G38"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1344,7 +1524,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1355,7 +1535,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1365,7 +1545,7 @@
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -1376,7 +1556,7 @@
     </row>
     <row r="5" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -1387,10 +1567,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
@@ -1399,11 +1579,11 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
-        <v>59</v>
+      <c r="A8" s="23" t="s">
+        <v>66</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -1412,11 +1592,11 @@
       <c r="G8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
-        <v>61</v>
+      <c r="A9" s="23" t="s">
+        <v>68</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
@@ -1425,11 +1605,11 @@
       <c r="G9" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
-        <v>63</v>
+      <c r="A10" s="23" t="s">
+        <v>70</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -1438,11 +1618,11 @@
       <c r="G10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
-        <v>65</v>
+      <c r="A11" s="23" t="s">
+        <v>72</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -1451,11 +1631,11 @@
       <c r="G11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
-        <v>67</v>
+      <c r="A12" s="23" t="s">
+        <v>74</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -1464,11 +1644,11 @@
       <c r="G12" s="7"/>
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
-        <v>69</v>
+      <c r="A13" s="23" t="s">
+        <v>76</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -1493,7 +1673,7 @@
     </row>
     <row r="16" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -1502,7 +1682,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -1516,7 +1696,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -1530,7 +1710,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -1544,7 +1724,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -1558,7 +1738,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -1572,7 +1752,7 @@
     </row>
     <row r="22" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -1586,7 +1766,7 @@
     </row>
     <row r="23" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -1600,7 +1780,7 @@
     </row>
     <row r="24" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -1614,7 +1794,7 @@
     </row>
     <row r="25" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -1648,30 +1828,80 @@
       <c r="F28" s="17"/>
       <c r="G28" s="17"/>
     </row>
-    <row r="30" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="19"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
+      <c r="F32" s="20"/>
+      <c r="G32" s="20"/>
+    </row>
+    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B33" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="22"/>
+    </row>
+    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+    </row>
+    <row r="36" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="27">
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="B7:G7"/>
@@ -1693,8 +1923,12 @@
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A26:G28"/>
-    <mergeCell ref="A30:G30"/>
-    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="B33:G33"/>
+    <mergeCell ref="B34:G34"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1711,7 +1945,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1722,7 +1956,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1732,7 +1966,7 @@
     </row>
     <row r="4" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -1743,7 +1977,7 @@
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -1754,58 +1988,58 @@
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1836,7 +2070,7 @@
     </row>
     <row r="17" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -1845,7 +2079,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -1859,7 +2093,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -1873,7 +2107,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -1887,7 +2121,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -1901,7 +2135,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -1915,7 +2149,7 @@
     </row>
     <row r="23" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -1929,7 +2163,7 @@
     </row>
     <row r="24" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -1943,7 +2177,7 @@
     </row>
     <row r="25" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -1957,7 +2191,7 @@
     </row>
     <row r="26" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -1991,30 +2225,80 @@
       <c r="F29" s="17"/>
       <c r="G29" s="17"/>
     </row>
-    <row r="31" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
+    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
+      <c r="G30" s="19"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="20"/>
+    </row>
+    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+    </row>
+    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="B35" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="C35" s="22"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="22"/>
+    </row>
+    <row r="37" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="21">
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A14:G14"/>
@@ -2030,8 +2314,12 @@
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A27:G29"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="B34:G34"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A38:G38"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2048,7 +2336,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -2059,7 +2347,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2069,7 +2357,7 @@
     </row>
     <row r="4" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -2080,7 +2368,7 @@
     </row>
     <row r="5" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -2091,10 +2379,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
@@ -2103,11 +2391,11 @@
       <c r="G7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
-        <v>113</v>
+      <c r="A8" s="23" t="s">
+        <v>130</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -2116,11 +2404,11 @@
       <c r="G8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
-        <v>115</v>
+      <c r="A9" s="23" t="s">
+        <v>132</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
@@ -2129,11 +2417,11 @@
       <c r="G9" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
-        <v>117</v>
+      <c r="A10" s="23" t="s">
+        <v>134</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -2142,11 +2430,11 @@
       <c r="G10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
-        <v>119</v>
+      <c r="A11" s="23" t="s">
+        <v>136</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -2155,11 +2443,11 @@
       <c r="G11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
-        <v>121</v>
+      <c r="A12" s="23" t="s">
+        <v>138</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -2168,11 +2456,11 @@
       <c r="G12" s="7"/>
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
-        <v>123</v>
+      <c r="A13" s="23" t="s">
+        <v>140</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -2197,7 +2485,7 @@
     </row>
     <row r="16" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -2211,7 +2499,7 @@
     </row>
     <row r="17" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -2225,7 +2513,7 @@
     </row>
     <row r="18" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -2239,7 +2527,7 @@
     </row>
     <row r="19" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -2253,7 +2541,7 @@
     </row>
     <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -2287,30 +2575,80 @@
       <c r="F23" s="17"/>
       <c r="G23" s="17"/>
     </row>
-    <row r="25" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="B29" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="22"/>
+    </row>
+    <row r="31" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="22">
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="B7:G7"/>
@@ -2327,8 +2665,12 @@
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="A21:G23"/>
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A32:G32"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
2.6.8: tallsporbarhet i alle 30 kapitler, OK03 balanseoppgave og finansregnskap
</commit_message>
<xml_diff>
--- a/pensum/ma01/MA01_Klasseoppgaver_v5.xlsx
+++ b/pensum/ma01/MA01_Klasseoppgaver_v5.xlsx
@@ -215,7 +215,7 @@
     <t xml:space="preserve">Kort oppsummert: Reklame er bare én del av markedsføringen. Boka regner også produktutvikling, emballasje, frakt og distribusjon, veiledende pris og kampanjepris som markedsføring. Kapittel 3.5 samler virkemidlene i de fem P-ene: produkt, pris, plass, påvirkning og personal. Markedsføringsledelse er det overordnede ansvaret for å planlegge, iverksette og evaluere markedsarbeidet; i små bedrifter ligger det hos daglig leder.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fjell Elektro AS har startet: Mona Fjell er daglig leder og faglig ansvarlig, og har to montører. I budsjettet står 40 000 kr til markedsføring under andre driftskostnader, og Mona har tenkt å bruke dem på annonser i lokalavisa og i sosiale medier. «Da er markedsføringen ordnet», sier hun. Bedriften har ingen rammeavtaler ennå og 3 500 fakturerbare timer i året. Gå fram slik: plasser kundene i hovedmarked, finn hvilken P et tiltak hører til, og vurder Monas påstand mot bokas definisjon.</t>
+    <t xml:space="preserve">Fjell Elektro AS har startet: Mona Fjell er daglig leder og faglig ansvarlig, og har to montører. I budsjettet står 40 000 kr til markedsføring under andre driftskostnader, og Mona har tenkt å bruke dem på annonser i lokalavisa og i sosiale medier. «Da er markedsføringen ordnet», sier hun. Bedriften har ingen rammeavtaler ennå og 3 500 fakturerbare timer i året: 2 montører × 1 400 timer + Mona 700 timer. Gå fram slik: plasser kundene i hovedmarked, finn hvilken P et tiltak hører til, og vurder Monas påstand mot bokas definisjon.</t>
   </si>
   <si>
     <t xml:space="preserve">Forutsetning</t>
@@ -257,7 +257,7 @@
     <t xml:space="preserve">Kapasitet</t>
   </si>
   <si>
-    <t xml:space="preserve">3 500 fakturerbare timer i året</t>
+    <t xml:space="preserve">3 500 fakturerbare timer i året (2 montører × 1 400 + Mona 700)</t>
   </si>
   <si>
     <t xml:space="preserve">a)  Fem kunder har ringt Fjell første måned. Hvilke av dem hører til forbrukermarkedet? Svar ja eller nei for hver, og si hvilket hovedmarked de andre hører til.</t>
@@ -356,7 +356,7 @@
     <t xml:space="preserve">Fakta</t>
   </si>
   <si>
-    <t xml:space="preserve">3 anbud i fjor, 0 vunnet, teknisk best alle</t>
+    <t xml:space="preserve">22 borettslag i nedslagsfeltet; 3 anbud i fjor, 0 vunnet, teknisk best alle</t>
   </si>
   <si>
     <t xml:space="preserve">a)  Hvilke av de fem forslagene starter hos kunden, og ikke hos det Nordlys allerede har? Svar ja eller nei for hver.</t>
@@ -2034,7 +2034,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
         <v>109</v>
       </c>

</xml_diff>